<commit_message>
speed benchmark sheet: flat list layout with No EV/Neutral/Boosted/Custom columns; add Rotom-Wash; rename sheet
</commit_message>
<xml_diff>
--- a/myteam/teams.xlsx
+++ b/myteam/teams.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Speed" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Speed Benchmark" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Strategy" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Mega" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Uber" sheetId="4" state="visible" r:id="rId4"/>
@@ -485,312 +485,614 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Base</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>No EV</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Boosted</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>No EV</t>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Custom Pokemon</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>50</v>
-      </c>
-      <c r="B2" t="n">
-        <v>106</v>
-      </c>
-      <c r="C2" t="n">
-        <v>97</v>
-      </c>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Clefable No EV</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
+      <c r="E2" t="n">
+        <v>75</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>60</v>
-      </c>
-      <c r="B3" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>61 No EV</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>76</v>
+      </c>
       <c r="C3" t="inlineStr"/>
-      <c r="D3" t="n">
-        <v>75</v>
-      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>61</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>70 No EV</t>
+        </is>
       </c>
       <c r="B4" t="n">
-        <v>118</v>
+        <v>85</v>
       </c>
       <c r="C4" t="inlineStr"/>
-      <c r="D4" t="n">
-        <v>76</v>
-      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>70</v>
-      </c>
-      <c r="B5" t="n">
-        <v>128</v>
-      </c>
-      <c r="C5" t="n">
-        <v>117</v>
-      </c>
-      <c r="D5" t="n">
-        <v>85</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Heatran No EV</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="n">
+        <v>92</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>75</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>80 No EV</t>
+        </is>
       </c>
       <c r="B6" t="n">
-        <v>134</v>
+        <v>95</v>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>77</v>
-      </c>
-      <c r="B7" t="n">
-        <v>136</v>
-      </c>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Azumarill Neutral</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
-      <c r="D7" t="n">
-        <v>92</v>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="n">
+        <v>97</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>80</v>
-      </c>
-      <c r="B8" t="n">
-        <v>139</v>
-      </c>
-      <c r="C8" t="n">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Rotom-Wash No EV</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>90 No EV</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>105</v>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Landorus-T No EV</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="n">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Diancie Boosted</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="n">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>100 No EV</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>115</v>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>70 Neutral</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="n">
+        <v>117</v>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>61 Boosted</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="n">
+        <v>118</v>
+      </c>
+      <c r="E14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>80 Neutral</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="n">
         <v>127</v>
       </c>
-      <c r="D8" t="n">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>85</v>
-      </c>
-      <c r="B9" t="n">
-        <v>145</v>
-      </c>
-      <c r="C9" t="n">
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>70 Boosted</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="n">
+        <v>128</v>
+      </c>
+      <c r="E16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>85 Neutral</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="n">
         <v>132</v>
       </c>
-      <c r="D9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>88</v>
-      </c>
-      <c r="B10" t="n">
-        <v>148</v>
-      </c>
-      <c r="C10" t="n">
-        <v>135</v>
-      </c>
-      <c r="D10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>90</v>
-      </c>
-      <c r="B11" t="n">
-        <v>150</v>
-      </c>
-      <c r="C11" t="n">
-        <v>137</v>
-      </c>
-      <c r="D11" t="n">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>91</v>
-      </c>
-      <c r="B12" t="n">
-        <v>151</v>
-      </c>
-      <c r="C12" t="n">
-        <v>138</v>
-      </c>
-      <c r="D12" t="n">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>95</v>
-      </c>
-      <c r="B13" t="n">
-        <v>156</v>
-      </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>100</v>
-      </c>
-      <c r="B14" t="n">
-        <v>161</v>
-      </c>
-      <c r="C14" t="n">
-        <v>147</v>
-      </c>
-      <c r="D14" t="n">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>102</v>
-      </c>
-      <c r="B15" t="n">
-        <v>163</v>
-      </c>
-      <c r="C15" t="n">
-        <v>149</v>
-      </c>
-      <c r="D15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>105</v>
-      </c>
-      <c r="B16" t="n">
-        <v>167</v>
-      </c>
-      <c r="C16" t="n">
-        <v>152</v>
-      </c>
-      <c r="D16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>108</v>
-      </c>
-      <c r="B17" t="n">
-        <v>170</v>
-      </c>
-      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="n">
-        <v>110</v>
-      </c>
-      <c r="B18" t="n">
-        <v>172</v>
-      </c>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>75 Boosted</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
+      <c r="D18" t="n">
+        <v>134</v>
+      </c>
+      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" t="n">
-        <v>111</v>
-      </c>
-      <c r="B19" t="n">
-        <v>173</v>
-      </c>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Excadrill Neutral</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
+      <c r="E19" t="n">
+        <v>135</v>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
-        <v>113</v>
-      </c>
-      <c r="B20" t="n">
-        <v>176</v>
-      </c>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Heatran Boosted</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
+      <c r="E20" t="n">
+        <v>136</v>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" t="n">
-        <v>115</v>
-      </c>
-      <c r="B21" t="n">
-        <v>178</v>
-      </c>
-      <c r="C21" t="inlineStr"/>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>90 Neutral</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="n">
+        <v>137</v>
+      </c>
       <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" t="n">
-        <v>120</v>
-      </c>
-      <c r="B22" t="n">
-        <v>183</v>
-      </c>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Landorus-T Neutral</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
+      <c r="E22" t="n">
+        <v>138</v>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" t="n">
-        <v>130</v>
-      </c>
-      <c r="B23" t="n">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>80 Boosted</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="n">
+        <v>139</v>
+      </c>
+      <c r="E23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>85 Boosted</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="n">
+        <v>145</v>
+      </c>
+      <c r="E24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Rotom-Wash Boosted</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>100 Neutral</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="n">
+        <v>147</v>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Excadrill Boosted</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>102 Neutral</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="n">
+        <v>149</v>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>90 Boosted</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="n">
+        <v>150</v>
+      </c>
+      <c r="E29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Landorus-T Boosted</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="n">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>105 Neutral</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="n">
+        <v>152</v>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>95 Boosted</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="n">
+        <v>156</v>
+      </c>
+      <c r="E32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>100 Boosted</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>161</v>
+      </c>
+      <c r="E33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Garchomp Boosted</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>105 Boosted</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="n">
+        <v>167</v>
+      </c>
+      <c r="E35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Keldeo Boosted</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>110 Boosted</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="n">
+        <v>172</v>
+      </c>
+      <c r="E37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Thundurus Boosted</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="n">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Serperior Boosted</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="n">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>115 Boosted</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="n">
+        <v>178</v>
+      </c>
+      <c r="E40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>120 Boosted</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="n">
+        <v>183</v>
+      </c>
+      <c r="E41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>130 Boosted</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="n">
         <v>194</v>
       </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>145</v>
-      </c>
-      <c r="B24" t="n">
+      <c r="E42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>150 Neutral</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="n">
+        <v>197</v>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>145 Boosted</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="n">
         <v>211</v>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>150</v>
-      </c>
-      <c r="B25" t="n">
+      <c r="E44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>150 Boosted</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="n">
         <v>216</v>
       </c>
-      <c r="C25" t="n">
-        <v>197</v>
-      </c>
-      <c r="D25" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
speed benchmark: fix stat formula (add +5 before nature); recompute all values at lv50/IV31
</commit_message>
<xml_diff>
--- a/myteam/teams.xlsx
+++ b/myteam/teams.xlsx
@@ -532,7 +532,7 @@
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3">
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
@@ -555,7 +555,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
@@ -571,7 +571,7 @@
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>92</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6">
@@ -581,7 +581,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
@@ -597,7 +597,7 @@
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
-        <v>97</v>
+        <v>102</v>
       </c>
     </row>
     <row r="8">
@@ -610,7 +610,7 @@
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
     </row>
     <row r="9">
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
@@ -636,7 +636,7 @@
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
-        <v>106</v>
+        <v>111</v>
       </c>
     </row>
     <row r="11">
@@ -649,7 +649,7 @@
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="12">
@@ -659,7 +659,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
@@ -673,7 +673,7 @@
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="n">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
@@ -687,7 +687,7 @@
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="n">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="E14" t="inlineStr"/>
     </row>
@@ -699,7 +699,7 @@
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="n">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
@@ -713,7 +713,7 @@
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="n">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E16" t="inlineStr"/>
     </row>
@@ -725,7 +725,7 @@
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="n">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
@@ -739,7 +739,7 @@
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="n">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="E18" t="inlineStr"/>
     </row>
@@ -753,7 +753,7 @@
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
-        <v>135</v>
+        <v>140</v>
       </c>
     </row>
     <row r="20">
@@ -766,7 +766,7 @@
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
-        <v>136</v>
+        <v>141</v>
       </c>
     </row>
     <row r="21">
@@ -777,7 +777,7 @@
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="n">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr"/>
@@ -792,7 +792,7 @@
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="n">
-        <v>138</v>
+        <v>143</v>
       </c>
     </row>
     <row r="23">
@@ -804,7 +804,7 @@
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="n">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="E23" t="inlineStr"/>
     </row>
@@ -817,7 +817,7 @@
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="n">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="E24" t="inlineStr"/>
     </row>
@@ -831,7 +831,7 @@
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="n">
-        <v>146</v>
+        <v>151</v>
       </c>
     </row>
     <row r="26">
@@ -842,7 +842,7 @@
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="n">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr"/>
@@ -850,28 +850,28 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Excadrill Boosted</t>
+          <t>102 Neutral</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
+      <c r="C27" t="n">
+        <v>154</v>
+      </c>
       <c r="D27" t="inlineStr"/>
-      <c r="E27" t="n">
-        <v>148</v>
-      </c>
+      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>102 Neutral</t>
+          <t>Excadrill Boosted</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
-      <c r="C28" t="n">
-        <v>149</v>
-      </c>
+      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="n">
+        <v>154</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -882,35 +882,35 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="n">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Landorus-T Boosted</t>
+          <t>105 Neutral</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
+      <c r="C30" t="n">
+        <v>157</v>
+      </c>
       <c r="D30" t="inlineStr"/>
-      <c r="E30" t="n">
-        <v>151</v>
-      </c>
+      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>105 Neutral</t>
+          <t>Landorus-T Boosted</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
-      <c r="C31" t="n">
-        <v>152</v>
-      </c>
+      <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
+      <c r="E31" t="n">
+        <v>157</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -921,7 +921,7 @@
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="n">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="E32" t="inlineStr"/>
     </row>
@@ -934,7 +934,7 @@
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="n">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="E33" t="inlineStr"/>
     </row>
@@ -948,7 +948,7 @@
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="n">
-        <v>163</v>
+        <v>169</v>
       </c>
     </row>
     <row r="35">
@@ -960,7 +960,7 @@
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="n">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="E35" t="inlineStr"/>
     </row>
@@ -974,7 +974,7 @@
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="n">
-        <v>170</v>
+        <v>176</v>
       </c>
     </row>
     <row r="37">
@@ -986,7 +986,7 @@
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="n">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="E37" t="inlineStr"/>
     </row>
@@ -1000,7 +1000,7 @@
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="n">
-        <v>173</v>
+        <v>179</v>
       </c>
     </row>
     <row r="39">
@@ -1013,7 +1013,7 @@
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="n">
-        <v>176</v>
+        <v>181</v>
       </c>
     </row>
     <row r="40">
@@ -1025,7 +1025,7 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="n">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="E40" t="inlineStr"/>
     </row>
@@ -1038,7 +1038,7 @@
       <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="n">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="E41" t="inlineStr"/>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="n">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="E42" t="inlineStr"/>
     </row>
@@ -1063,7 +1063,7 @@
       </c>
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="n">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr"/>
@@ -1077,7 +1077,7 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="n">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="E44" t="inlineStr"/>
     </row>
@@ -1090,7 +1090,7 @@
       <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="n">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="E45" t="inlineStr"/>
     </row>

</xml_diff>